<commit_message>
README: replay results on real lines; workbook Replay sheet
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CfNTq3mdgKxDd9mNevjxAe
</commit_message>
<xml_diff>
--- a/data/exports/edgeline_model.xlsx
+++ b/data/exports/edgeline_model.xlsx
@@ -12,9 +12,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slips" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Line shopping" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Real-line record" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backtest" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graded lines" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Replay" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backtest" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graded lines" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Board'!$A$3:$O$515</definedName>
@@ -22,8 +23,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Slips'!$A$3:$N$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Line shopping'!$A$3:$Q$87</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Real-line record'!$A$3:$K$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Backtest'!$A$3:$L$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Graded lines'!$A$3:$M$430</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Replay'!$A$3:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Backtest'!$A$3:$L$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Graded lines'!$A$3:$M$430</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -47786,6 +47788,428 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Replay: models trained only on games before 2026-09-25, pointed at that day's real PrizePicks opening lines (out of sample on real lines).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>sport</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>slice</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>wins</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>losses</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>hit rate</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>CI low</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>CI high</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>4-pick ROI</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>dota</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>all leans</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>0.6964285714285714</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>0.5666413460816312</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>0.8009967498351162</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>1.352373726116722</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>dota</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>bettable</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>0.4385029643606804</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>dota</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>kills leans</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>0.6964285714285714</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>0.5666413460816312</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>0.8009967498351162</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>1.352373726116722</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>lol</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>all leans</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>0.7826086956521739</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>0.5809651681324879</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>0.9033602203455142</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>2.751273044335892</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>lol</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>bettable</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>0.7692307692307693</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>0.4974362383948036</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>0.918204713457304</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>2.501277966457758</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>lol</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>kills leans</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>0.7826086956521739</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>0.5809651681324879</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>0.9033602203455142</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>2.751273044335892</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>cs2</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>all leans</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>378</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>178</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>0.5291005291005291</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>0.4787412738024508</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>0.5788742613582798</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>-0.216294700891745</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>cs2</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>bettable</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>0.5806451612903226</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>0.4076626236738884</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>0.7358445703570756</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>0.1366931558675983</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>cs2</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>headshots leans</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>168</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>97</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>71</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>0.5773809523809523</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>0.5017741756089368</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>0.6495280780454632</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>0.1113473292579026</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>cs2</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>kills leans</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>210</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>103</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>107</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>0.4904761904761905</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>0.4236441973629771</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>0.5576503559901199</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>-0.4212756978830838</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:I13"/>
+  <conditionalFormatting sqref="F4:F13">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0.45"/>
+        <cfvo type="num" val="0.5623"/>
+        <cfvo type="num" val="0.7"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFFFFF"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -48855,7 +49279,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -74166,7 +74590,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Workbook: match counts and match-cluster interval on the real-line record sheet
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CfNTq3mdgKxDd9mNevjxAe
</commit_message>
<xml_diff>
--- a/data/exports/edgeline_model.xlsx
+++ b/data/exports/edgeline_model.xlsx
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Slips'!$A$3:$N$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Stacks'!$A$3:$N$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Line shopping'!$A$3:$Q$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Real-line record'!$A$3:$K$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Real-line record'!$A$3:$O$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Closing-line value'!$A$3:$H$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Replay'!$A$3:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Stack backtest'!$A$3:$M$37</definedName>
@@ -602,7 +602,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Edgeline board: every upcoming PrizePicks line priced by the model (as of 2026-09-26 10:07 UTC). Green rows = bettable (&gt;= 60% probability and &gt;= 5% EV, standard odds, not voidable, not moved &gt; 10% against).</t>
+          <t>Edgeline board: every upcoming PrizePicks line priced by the model (as of 2026-09-26 10:10 UTC). Green rows = bettable (&gt;= 60% probability and &gt;= 5% EV, standard odds, not voidable, not moved &gt; 10% against).</t>
         </is>
       </c>
     </row>
@@ -74999,7 +74999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -75013,12 +75013,16 @@
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="23" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Captured PrizePicks opening lines graded against results (edgeline roi). Break-even for a 4-pick power is 56.2% per leg; the 30% ROI target is 60%. Green = the 95% interval's lower bound clears the bar.</t>
+          <t>Captured PrizePicks opening lines graded against results (edgeline roi). Break-even for a 4-pick power is 56.2% per leg; the 30% ROI target is 60%. Lines from one match win or lose together, so the match-cluster interval (unordered team pair + day, needs 5+ matches) is the one that proves a market. Green = the interval's lower bound clears the bar.</t>
         </is>
       </c>
     </row>
@@ -75078,6 +75082,26 @@
           <t>above 60% target</t>
         </is>
       </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>matches</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>match-cluster CI low</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>match-cluster CI high</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>proven by matches</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -75119,6 +75143,20 @@
           <t>no</t>
         </is>
       </c>
+      <c r="L4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="M4" s="6" t="n">
+        <v>0.4720174474899448</v>
+      </c>
+      <c r="N4" s="6" t="n">
+        <v>0.6218202479338842</v>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -75160,6 +75198,20 @@
           <t>no</t>
         </is>
       </c>
+      <c r="L5" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>0.3636034255599473</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>0.7342051377513029</v>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -75201,6 +75253,20 @@
           <t>no</t>
         </is>
       </c>
+      <c r="L6" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="M6" s="6" t="n">
+        <v>0.4197961127308066</v>
+      </c>
+      <c r="N6" s="6" t="n">
+        <v>0.5888975448536354</v>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -75242,6 +75308,20 @@
           <t>no</t>
         </is>
       </c>
+      <c r="L7" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>0.2999675324675324</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>0.6481606606606606</v>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -75283,6 +75363,20 @@
           <t>no</t>
         </is>
       </c>
+      <c r="L8" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="M8" s="6" t="n">
+        <v>0.4838602862636189</v>
+      </c>
+      <c r="N8" s="6" t="n">
+        <v>0.6496894904458598</v>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -75324,6 +75418,20 @@
           <t>no</t>
         </is>
       </c>
+      <c r="L9" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>0.3405619494174482</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>0.5571146488954706</v>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -75365,6 +75473,20 @@
           <t>no</t>
         </is>
       </c>
+      <c r="L10" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="M10" s="6" t="n">
+        <v>0.3295305023923445</v>
+      </c>
+      <c r="N10" s="6" t="n">
+        <v>0.5384615384615384</v>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -75406,6 +75528,20 @@
           <t>no</t>
         </is>
       </c>
+      <c r="L11" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>0.4391474538533362</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>0.6375572263004182</v>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -75447,6 +75583,16 @@
           <t>no</t>
         </is>
       </c>
+      <c r="L12" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M12" s="6" t="n"/>
+      <c r="N12" s="6" t="n"/>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>too few matches</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -75488,6 +75634,16 @@
           <t>no</t>
         </is>
       </c>
+      <c r="L13" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M13" s="6" t="n"/>
+      <c r="N13" s="6" t="n"/>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>too few matches</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -75529,6 +75685,16 @@
           <t>no</t>
         </is>
       </c>
+      <c r="L14" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M14" s="6" t="n"/>
+      <c r="N14" s="6" t="n"/>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>too few matches</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -75570,6 +75736,16 @@
           <t>no</t>
         </is>
       </c>
+      <c r="L15" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M15" s="6" t="n"/>
+      <c r="N15" s="6" t="n"/>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>too few matches</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -75611,6 +75787,16 @@
           <t>YES</t>
         </is>
       </c>
+      <c r="L16" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M16" s="6" t="n"/>
+      <c r="N16" s="6" t="n"/>
+      <c r="O16" s="4" t="inlineStr">
+        <is>
+          <t>too few matches</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -75652,6 +75838,16 @@
           <t>no</t>
         </is>
       </c>
+      <c r="L17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" s="6" t="n"/>
+      <c r="N17" s="6" t="n"/>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>too few matches</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -75693,6 +75889,16 @@
           <t>YES</t>
         </is>
       </c>
+      <c r="L18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="6" t="n"/>
+      <c r="N18" s="6" t="n"/>
+      <c r="O18" s="4" t="inlineStr">
+        <is>
+          <t>too few matches</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -75734,6 +75940,16 @@
           <t>no</t>
         </is>
       </c>
+      <c r="L19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" s="6" t="n"/>
+      <c r="N19" s="6" t="n"/>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>too few matches</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -75775,6 +75991,16 @@
           <t>no</t>
         </is>
       </c>
+      <c r="L20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M20" s="6" t="n"/>
+      <c r="N20" s="6" t="n"/>
+      <c r="O20" s="4" t="inlineStr">
+        <is>
+          <t>too few matches</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -75816,6 +76042,16 @@
           <t>no</t>
         </is>
       </c>
+      <c r="L21" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" s="6" t="n"/>
+      <c r="N21" s="6" t="n"/>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>too few matches</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -75857,9 +76093,19 @@
           <t>YES</t>
         </is>
       </c>
+      <c r="L22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" s="6" t="n"/>
+      <c r="N22" s="6" t="n"/>
+      <c r="O22" s="4" t="inlineStr">
+        <is>
+          <t>too few matches</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:K22"/>
+  <autoFilter ref="A3:O22"/>
   <conditionalFormatting sqref="J4:J22">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"YES"</formula>
@@ -75870,8 +76116,13 @@
       <formula>"YES"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="O4:O22">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="0">
+      <formula>"YES"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="E4:E22">
-    <cfRule type="colorScale" priority="3">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="num" val="0.45"/>
         <cfvo type="num" val="0.5623"/>
@@ -76129,10 +76380,10 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="D10" s="4" t="n">
         <v>13</v>
@@ -76147,7 +76398,7 @@
         <v>0.3833103179931641</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>0.004914004914004914</v>
+        <v>0.004926108374384237</v>
       </c>
     </row>
     <row r="11">
@@ -76157,10 +76408,10 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D11" s="4" t="n">
         <v>17</v>
@@ -76175,7 +76426,7 @@
         <v>0.000728607177734375</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>0.06331877729257641</v>
+        <v>0.06304347826086956</v>
       </c>
     </row>
     <row r="12">

</xml_diff>